<commit_message>
Filter SO line items by active SKUs; remove retired SKUs from template and row mapping
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bertrandnicoli/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bertrandnicoli/belfast_RPA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87FCBF29-07D2-7148-8C8A-0F8193B0ABED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8792BFD0-7389-5A4B-93B1-05CCBBF128EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -530,9 +530,6 @@
     <t>Cert Number</t>
   </si>
   <si>
-    <t>BOSH0090</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <u/>
@@ -544,9 +541,6 @@
     </r>
   </si>
   <si>
-    <t>BOSH! Spicy No-Duja Sourdough Pizza - 275g</t>
-  </si>
-  <si>
     <t>Case</t>
   </si>
   <si>
@@ -554,15 +548,6 @@
   </si>
   <si>
     <t>NIRMS</t>
-  </si>
-  <si>
-    <t>BOSH0089</t>
-  </si>
-  <si>
-    <t>BOSH! Margherita Sourdough Pizza - 275g</t>
-  </si>
-  <si>
-    <t>BOSH0082</t>
   </si>
   <si>
     <r>
@@ -576,9 +561,6 @@
     </r>
   </si>
   <si>
-    <t>BOSH! Hearty Vegetable Lasagne 380g</t>
-  </si>
-  <si>
     <t>BOSH0077</t>
   </si>
   <si>
@@ -591,12 +573,6 @@
     <t>BOSH! Creamy Mac &amp; Greens 380g</t>
   </si>
   <si>
-    <t>BOSH0081</t>
-  </si>
-  <si>
-    <t>BOSH! Ultimate Bean Chilli 380g</t>
-  </si>
-  <si>
     <t>BOSH0080</t>
   </si>
   <si>
@@ -604,13 +580,38 @@
   </si>
   <si>
     <t>GB</t>
+  </si>
+  <si>
+    <t>BOSH0101</t>
+  </si>
+  <si>
+    <t>BOSH! Peanut Satay Noodles</t>
+  </si>
+  <si>
+    <t>BOSH0102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	
+BOSH! Katsu Curry</t>
+  </si>
+  <si>
+    <t>BOSH0103</t>
+  </si>
+  <si>
+    <t>BOSH0104</t>
+  </si>
+  <si>
+    <t>BOSH! Pepper-Noni Pizza 10 Inch</t>
+  </si>
+  <si>
+    <t>BOSH! Margherita Pizza - 10 Inch</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -804,6 +805,12 @@
       <color rgb="FF1155CC"/>
       <name val="Calibri, sans-serif"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -914,7 +921,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1053,6 +1060,9 @@
     </xf>
     <xf numFmtId="15" fontId="11" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1285,7 +1295,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:S999"/>
+  <dimension ref="A1:S995"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="4" max="4" width="17.6640625" customWidth="1"/>
@@ -1298,18 +1308,18 @@
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="2"/>
@@ -1368,7 +1378,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="8"/>
-      <c r="D4" s="57" t="s">
+      <c r="D4" s="58" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="5" t="s">
@@ -1399,18 +1409,18 @@
         <v>8</v>
       </c>
       <c r="C5" s="13"/>
-      <c r="D5" s="58"/>
+      <c r="D5" s="59"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="6"/>
-      <c r="K5" s="61" t="s">
+      <c r="K5" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="58"/>
-      <c r="M5" s="58"/>
+      <c r="L5" s="59"/>
+      <c r="M5" s="59"/>
       <c r="N5" s="15"/>
       <c r="O5" s="15"/>
       <c r="P5" s="15"/>
@@ -1426,7 +1436,7 @@
       <c r="C6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="58"/>
+      <c r="D6" s="59"/>
       <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1435,10 +1445,10 @@
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
       <c r="J6" s="9"/>
-      <c r="K6" s="61" t="s">
+      <c r="K6" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="58"/>
+      <c r="L6" s="59"/>
       <c r="M6" s="15"/>
       <c r="N6" s="15"/>
       <c r="O6" s="15"/>
@@ -1453,7 +1463,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="9"/>
-      <c r="D7" s="58"/>
+      <c r="D7" s="59"/>
       <c r="E7" s="5" t="s">
         <v>15</v>
       </c>
@@ -1462,10 +1472,10 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
       <c r="J7" s="16"/>
-      <c r="K7" s="61" t="s">
+      <c r="K7" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="L7" s="58"/>
+      <c r="L7" s="59"/>
       <c r="M7" s="15"/>
       <c r="N7" s="15"/>
       <c r="O7" s="15"/>
@@ -1480,7 +1490,7 @@
         <v>17</v>
       </c>
       <c r="C8" s="9"/>
-      <c r="D8" s="58"/>
+      <c r="D8" s="59"/>
       <c r="E8" s="5" t="s">
         <v>18</v>
       </c>
@@ -1491,11 +1501,11 @@
       <c r="H8" s="10"/>
       <c r="I8" s="10"/>
       <c r="J8" s="17"/>
-      <c r="K8" s="61" t="s">
+      <c r="K8" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="L8" s="58"/>
-      <c r="M8" s="58"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
       <c r="P8" s="15"/>
@@ -1504,14 +1514,14 @@
       <c r="S8" s="3"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="58" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C9" s="16"/>
-      <c r="D9" s="58"/>
+      <c r="D9" s="59"/>
       <c r="E9" s="5" t="s">
         <v>23</v>
       </c>
@@ -1531,12 +1541,12 @@
       <c r="S9" s="3"/>
     </row>
     <row r="10" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A10" s="58"/>
+      <c r="A10" s="59"/>
       <c r="B10" s="5" t="s">
         <v>24</v>
       </c>
       <c r="C10" s="16"/>
-      <c r="D10" s="58"/>
+      <c r="D10" s="59"/>
       <c r="E10" s="5" t="s">
         <v>25</v>
       </c>
@@ -1560,14 +1570,14 @@
       <c r="S10" s="3"/>
     </row>
     <row r="11" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A11" s="58"/>
+      <c r="A11" s="59"/>
       <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C11" s="17">
         <v>3</v>
       </c>
-      <c r="D11" s="58"/>
+      <c r="D11" s="59"/>
       <c r="E11" s="5" t="s">
         <v>29</v>
       </c>
@@ -1589,12 +1599,12 @@
       <c r="S11" s="3"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A12" s="58"/>
+      <c r="A12" s="59"/>
       <c r="B12" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C12" s="17"/>
-      <c r="D12" s="58"/>
+      <c r="D12" s="59"/>
       <c r="E12" s="5" t="s">
         <v>30</v>
       </c>
@@ -1624,26 +1634,26 @@
         <v>37</v>
       </c>
       <c r="Q12" s="3"/>
-      <c r="R12" s="59" t="s">
+      <c r="R12" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="S12" s="58"/>
+      <c r="S12" s="59"/>
     </row>
     <row r="13" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A13" s="58"/>
+      <c r="A13" s="59"/>
       <c r="B13" s="5" t="s">
         <v>39</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="58"/>
+      <c r="D13" s="59"/>
       <c r="E13" s="5" t="s">
         <v>41</v>
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="19"/>
-      <c r="H13" s="57" t="s">
+      <c r="H13" s="58" t="s">
         <v>42</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -1663,24 +1673,24 @@
       <c r="S13" s="3"/>
     </row>
     <row r="14" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A14" s="58"/>
+      <c r="A14" s="59"/>
       <c r="B14" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C14" s="17"/>
-      <c r="D14" s="58"/>
+      <c r="D14" s="59"/>
       <c r="E14" s="5" t="s">
         <v>46</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="19"/>
-      <c r="H14" s="58"/>
+      <c r="H14" s="59"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="62" t="s">
+      <c r="J14" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="K14" s="58"/>
-      <c r="L14" s="58"/>
+      <c r="K14" s="59"/>
+      <c r="L14" s="59"/>
       <c r="M14" s="20" t="s">
         <v>48</v>
       </c>
@@ -1692,14 +1702,14 @@
       <c r="S14" s="3"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A15" s="58"/>
+      <c r="A15" s="59"/>
       <c r="B15" s="5" t="s">
         <v>49</v>
       </c>
       <c r="C15" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="58"/>
+      <c r="D15" s="59"/>
       <c r="E15" s="5" t="s">
         <v>51</v>
       </c>
@@ -1707,7 +1717,7 @@
         <v>52</v>
       </c>
       <c r="G15" s="19"/>
-      <c r="H15" s="58"/>
+      <c r="H15" s="59"/>
       <c r="I15" s="2"/>
       <c r="J15" s="22"/>
       <c r="K15" s="22"/>
@@ -1723,12 +1733,12 @@
       <c r="S15" s="3"/>
     </row>
     <row r="16" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A16" s="58"/>
+      <c r="A16" s="59"/>
       <c r="B16" s="23" t="s">
         <v>54</v>
       </c>
       <c r="C16" s="17"/>
-      <c r="D16" s="58"/>
+      <c r="D16" s="59"/>
       <c r="E16" s="5" t="s">
         <v>55</v>
       </c>
@@ -1736,7 +1746,7 @@
         <v>56</v>
       </c>
       <c r="G16" s="19"/>
-      <c r="H16" s="58"/>
+      <c r="H16" s="59"/>
       <c r="I16" s="2"/>
       <c r="J16" s="22"/>
       <c r="K16" s="22"/>
@@ -1752,16 +1762,16 @@
       <c r="S16" s="3"/>
     </row>
     <row r="17" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A17" s="58"/>
+      <c r="A17" s="59"/>
       <c r="B17" s="5"/>
       <c r="C17" s="22"/>
-      <c r="D17" s="58"/>
+      <c r="D17" s="59"/>
       <c r="E17" s="5"/>
       <c r="F17" s="24" t="s">
         <v>58</v>
       </c>
       <c r="G17" s="19"/>
-      <c r="H17" s="58"/>
+      <c r="H17" s="59"/>
       <c r="I17" s="2"/>
       <c r="J17" s="22"/>
       <c r="K17" s="22"/>
@@ -1777,18 +1787,18 @@
       <c r="S17" s="3"/>
     </row>
     <row r="18" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A18" s="58"/>
+      <c r="A18" s="59"/>
       <c r="B18" s="25" t="s">
         <v>60</v>
       </c>
       <c r="C18" s="22"/>
-      <c r="D18" s="58"/>
+      <c r="D18" s="59"/>
       <c r="E18" s="25" t="s">
         <v>61</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="19"/>
-      <c r="H18" s="58"/>
+      <c r="H18" s="59"/>
       <c r="I18" s="3"/>
       <c r="J18" s="18" t="s">
         <v>32</v>
@@ -1808,12 +1818,12 @@
       <c r="S18" s="3"/>
     </row>
     <row r="19" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A19" s="58"/>
+      <c r="A19" s="59"/>
       <c r="B19" s="5" t="s">
         <v>62</v>
       </c>
       <c r="C19" s="27"/>
-      <c r="D19" s="58"/>
+      <c r="D19" s="59"/>
       <c r="E19" s="28" t="s">
         <v>63</v>
       </c>
@@ -1821,7 +1831,7 @@
         <v>64</v>
       </c>
       <c r="G19" s="19"/>
-      <c r="H19" s="58"/>
+      <c r="H19" s="59"/>
       <c r="I19" s="5" t="s">
         <v>65</v>
       </c>
@@ -1839,22 +1849,22 @@
       <c r="S19" s="3"/>
     </row>
     <row r="20" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A20" s="58"/>
+      <c r="A20" s="59"/>
       <c r="B20" s="5" t="s">
         <v>66</v>
       </c>
       <c r="C20" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="D20" s="58"/>
+      <c r="D20" s="59"/>
       <c r="E20" s="5" t="s">
         <v>68</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="G20" s="19"/>
-      <c r="H20" s="58"/>
+      <c r="H20" s="59"/>
       <c r="I20" s="2"/>
       <c r="J20" s="22"/>
       <c r="K20" s="22"/>
@@ -1870,18 +1880,18 @@
       <c r="S20" s="3"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A21" s="58"/>
+      <c r="A21" s="59"/>
       <c r="B21" s="5" t="s">
         <v>70</v>
       </c>
       <c r="C21" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="D21" s="58"/>
+      <c r="D21" s="59"/>
       <c r="E21" s="19"/>
       <c r="F21" s="19"/>
       <c r="G21" s="19"/>
-      <c r="H21" s="58"/>
+      <c r="H21" s="59"/>
       <c r="I21" s="3"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
@@ -1895,18 +1905,18 @@
       <c r="S21" s="2"/>
     </row>
     <row r="22" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A22" s="58"/>
+      <c r="A22" s="59"/>
       <c r="B22" s="5" t="s">
         <v>72</v>
       </c>
       <c r="C22" s="30"/>
-      <c r="D22" s="58"/>
+      <c r="D22" s="59"/>
       <c r="E22" s="5" t="s">
         <v>73</v>
       </c>
       <c r="F22" s="27"/>
       <c r="G22" s="19"/>
-      <c r="H22" s="58"/>
+      <c r="H22" s="59"/>
       <c r="I22" s="5" t="s">
         <v>74</v>
       </c>
@@ -1924,14 +1934,14 @@
       <c r="S22" s="2"/>
     </row>
     <row r="23" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A23" s="58"/>
+      <c r="A23" s="59"/>
       <c r="B23" s="5" t="s">
         <v>75</v>
       </c>
       <c r="C23" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="58"/>
+      <c r="D23" s="59"/>
       <c r="E23" s="5" t="s">
         <v>77</v>
       </c>
@@ -1939,7 +1949,7 @@
         <v>11</v>
       </c>
       <c r="G23" s="19"/>
-      <c r="H23" s="58"/>
+      <c r="H23" s="59"/>
       <c r="I23" s="2"/>
       <c r="J23" s="22"/>
       <c r="K23" s="22"/>
@@ -1955,12 +1965,12 @@
       <c r="S23" s="2"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A24" s="58"/>
+      <c r="A24" s="59"/>
       <c r="B24" s="5" t="s">
         <v>78</v>
       </c>
       <c r="C24" s="30"/>
-      <c r="D24" s="58"/>
+      <c r="D24" s="59"/>
       <c r="E24" s="5" t="s">
         <v>79</v>
       </c>
@@ -1968,7 +1978,7 @@
         <v>80</v>
       </c>
       <c r="G24" s="19"/>
-      <c r="H24" s="58"/>
+      <c r="H24" s="59"/>
       <c r="I24" s="3"/>
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
@@ -1982,14 +1992,14 @@
       <c r="S24" s="2"/>
     </row>
     <row r="25" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A25" s="58"/>
+      <c r="A25" s="59"/>
       <c r="B25" s="5" t="s">
         <v>81</v>
       </c>
       <c r="C25" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="D25" s="58"/>
+      <c r="D25" s="59"/>
       <c r="E25" s="5" t="s">
         <v>83</v>
       </c>
@@ -1997,7 +2007,7 @@
         <v>84</v>
       </c>
       <c r="G25" s="19"/>
-      <c r="H25" s="58"/>
+      <c r="H25" s="59"/>
       <c r="I25" s="5" t="s">
         <v>74</v>
       </c>
@@ -2015,10 +2025,10 @@
       <c r="S25" s="2"/>
     </row>
     <row r="26" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A26" s="58"/>
+      <c r="A26" s="59"/>
       <c r="B26" s="19"/>
       <c r="C26" s="19"/>
-      <c r="D26" s="58"/>
+      <c r="D26" s="59"/>
       <c r="E26" s="5" t="s">
         <v>85</v>
       </c>
@@ -2026,7 +2036,7 @@
         <v>86</v>
       </c>
       <c r="G26" s="19"/>
-      <c r="H26" s="58"/>
+      <c r="H26" s="59"/>
       <c r="I26" s="2"/>
       <c r="J26" s="22"/>
       <c r="K26" s="22"/>
@@ -2042,12 +2052,12 @@
       <c r="S26" s="2"/>
     </row>
     <row r="27" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A27" s="58"/>
+      <c r="A27" s="59"/>
       <c r="B27" s="5" t="s">
         <v>87</v>
       </c>
       <c r="C27" s="17"/>
-      <c r="D27" s="58"/>
+      <c r="D27" s="59"/>
       <c r="E27" s="5" t="s">
         <v>88</v>
       </c>
@@ -2055,7 +2065,7 @@
         <v>86</v>
       </c>
       <c r="G27" s="19"/>
-      <c r="H27" s="58"/>
+      <c r="H27" s="59"/>
       <c r="I27" s="3"/>
       <c r="J27" s="18"/>
       <c r="K27" s="18"/>
@@ -2069,12 +2079,12 @@
       <c r="S27" s="2"/>
     </row>
     <row r="28" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A28" s="58"/>
+      <c r="A28" s="59"/>
       <c r="B28" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C28" s="17"/>
-      <c r="D28" s="58"/>
+      <c r="D28" s="59"/>
       <c r="E28" s="5" t="s">
         <v>90</v>
       </c>
@@ -2082,7 +2092,7 @@
         <v>91</v>
       </c>
       <c r="G28" s="19"/>
-      <c r="H28" s="58"/>
+      <c r="H28" s="59"/>
       <c r="I28" s="5" t="s">
         <v>74</v>
       </c>
@@ -2100,16 +2110,16 @@
       <c r="S28" s="2"/>
     </row>
     <row r="29" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A29" s="58"/>
+      <c r="A29" s="59"/>
       <c r="B29" s="5" t="s">
         <v>92</v>
       </c>
       <c r="C29" s="17"/>
-      <c r="D29" s="58"/>
+      <c r="D29" s="59"/>
       <c r="E29" s="19"/>
       <c r="F29" s="19"/>
       <c r="G29" s="19"/>
-      <c r="H29" s="58"/>
+      <c r="H29" s="59"/>
       <c r="I29" s="2"/>
       <c r="J29" s="22"/>
       <c r="K29" s="22"/>
@@ -2125,16 +2135,16 @@
       <c r="S29" s="2"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A30" s="58"/>
+      <c r="A30" s="59"/>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
-      <c r="D30" s="58"/>
+      <c r="D30" s="59"/>
       <c r="E30" s="25" t="s">
         <v>93</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="19"/>
-      <c r="H30" s="58"/>
+      <c r="H30" s="59"/>
       <c r="I30" s="3"/>
       <c r="J30" s="18" t="s">
         <v>32</v>
@@ -2154,18 +2164,18 @@
       <c r="S30" s="2"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A31" s="58"/>
+      <c r="A31" s="59"/>
       <c r="B31" s="25" t="s">
         <v>94</v>
       </c>
       <c r="C31" s="22"/>
-      <c r="D31" s="58"/>
+      <c r="D31" s="59"/>
       <c r="E31" s="28" t="s">
         <v>95</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="19"/>
-      <c r="H31" s="58"/>
+      <c r="H31" s="59"/>
       <c r="I31" s="5" t="s">
         <v>96</v>
       </c>
@@ -2183,12 +2193,12 @@
       <c r="S31" s="2"/>
     </row>
     <row r="32" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A32" s="58"/>
+      <c r="A32" s="59"/>
       <c r="B32" s="5" t="s">
         <v>97</v>
       </c>
       <c r="C32" s="17"/>
-      <c r="D32" s="58"/>
+      <c r="D32" s="59"/>
       <c r="E32" s="5" t="s">
         <v>98</v>
       </c>
@@ -2196,11 +2206,11 @@
       <c r="G32" s="19"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="62" t="s">
+      <c r="J32" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="K32" s="58"/>
-      <c r="L32" s="58"/>
+      <c r="K32" s="59"/>
+      <c r="L32" s="59"/>
       <c r="M32" s="20" t="s">
         <v>99</v>
       </c>
@@ -2212,14 +2222,14 @@
       <c r="S32" s="2"/>
     </row>
     <row r="33" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A33" s="58"/>
+      <c r="A33" s="59"/>
       <c r="B33" s="5" t="s">
         <v>100</v>
       </c>
       <c r="C33" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="D33" s="58"/>
+      <c r="D33" s="59"/>
       <c r="E33" s="19"/>
       <c r="F33" s="19"/>
       <c r="G33" s="19"/>
@@ -2239,14 +2249,14 @@
       <c r="S33" s="2"/>
     </row>
     <row r="34" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A34" s="58"/>
+      <c r="A34" s="59"/>
       <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
       <c r="C34" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="58"/>
+      <c r="D34" s="59"/>
       <c r="E34" s="5" t="s">
         <v>105</v>
       </c>
@@ -2268,12 +2278,12 @@
       <c r="S34" s="2"/>
     </row>
     <row r="35" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A35" s="58"/>
+      <c r="A35" s="59"/>
       <c r="B35" s="5" t="s">
         <v>107</v>
       </c>
       <c r="C35" s="31"/>
-      <c r="D35" s="58"/>
+      <c r="D35" s="59"/>
       <c r="E35" s="5" t="s">
         <v>108</v>
       </c>
@@ -2297,14 +2307,14 @@
       <c r="S35" s="2"/>
     </row>
     <row r="36" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A36" s="58"/>
+      <c r="A36" s="59"/>
       <c r="B36" s="5" t="s">
         <v>111</v>
       </c>
       <c r="C36" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="D36" s="58"/>
+      <c r="D36" s="59"/>
       <c r="E36" s="5" t="s">
         <v>113</v>
       </c>
@@ -2326,14 +2336,14 @@
       <c r="S36" s="2"/>
     </row>
     <row r="37" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A37" s="58"/>
+      <c r="A37" s="59"/>
       <c r="B37" s="5" t="s">
         <v>115</v>
       </c>
       <c r="C37" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="D37" s="58"/>
+      <c r="D37" s="59"/>
       <c r="E37" s="5" t="s">
         <v>117</v>
       </c>
@@ -2355,14 +2365,14 @@
       <c r="S37" s="2"/>
     </row>
     <row r="38" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A38" s="58"/>
+      <c r="A38" s="59"/>
       <c r="B38" s="5" t="s">
         <v>119</v>
       </c>
       <c r="C38" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="D38" s="58"/>
+      <c r="D38" s="59"/>
       <c r="E38" s="5" t="s">
         <v>121</v>
       </c>
@@ -2373,10 +2383,10 @@
         <v>122</v>
       </c>
       <c r="J38" s="36"/>
-      <c r="K38" s="63" t="s">
+      <c r="K38" s="64" t="s">
         <v>123</v>
       </c>
-      <c r="L38" s="58"/>
+      <c r="L38" s="59"/>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -2386,10 +2396,10 @@
       <c r="S38" s="2"/>
     </row>
     <row r="39" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A39" s="58"/>
+      <c r="A39" s="59"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
-      <c r="D39" s="58"/>
+      <c r="D39" s="59"/>
       <c r="E39" s="5" t="s">
         <v>124</v>
       </c>
@@ -2411,7 +2421,7 @@
       <c r="S39" s="2"/>
     </row>
     <row r="40" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A40" s="58"/>
+      <c r="A40" s="59"/>
       <c r="B40" s="5" t="s">
         <v>126</v>
       </c>
@@ -2436,7 +2446,7 @@
       <c r="S40" s="2"/>
     </row>
     <row r="41" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A41" s="58"/>
+      <c r="A41" s="59"/>
       <c r="B41" s="5" t="s">
         <v>128</v>
       </c>
@@ -2461,7 +2471,7 @@
       <c r="S41" s="2"/>
     </row>
     <row r="42" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A42" s="58"/>
+      <c r="A42" s="59"/>
       <c r="B42" s="5" t="s">
         <v>129</v>
       </c>
@@ -2603,26 +2613,24 @@
         <v>1</v>
       </c>
       <c r="B46" s="45" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C46" s="46">
         <v>2106909869</v>
       </c>
       <c r="D46" s="47" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E46" s="20"/>
       <c r="F46" s="48" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G46" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="H46" s="52">
-        <v>5</v>
-      </c>
+      <c r="H46" s="52"/>
       <c r="I46" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J46" s="16">
         <v>1.7909999999999999</v>
@@ -2637,10 +2645,10 @@
         <v>40</v>
       </c>
       <c r="N46" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O46" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P46" s="48" t="s">
         <v>52</v>
@@ -2654,26 +2662,24 @@
         <v>2</v>
       </c>
       <c r="B47" s="45" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C47" s="46">
         <v>2106909869</v>
       </c>
       <c r="D47" s="47" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E47" s="20"/>
       <c r="F47" s="48" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="G47" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="H47" s="52">
-        <v>6</v>
-      </c>
+      <c r="H47" s="52"/>
       <c r="I47" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J47" s="16">
         <v>1.7909999999999999</v>
@@ -2688,10 +2694,10 @@
         <v>40</v>
       </c>
       <c r="N47" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O47" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P47" s="48" t="s">
         <v>52</v>
@@ -2705,26 +2711,24 @@
         <v>3</v>
       </c>
       <c r="B48" s="45" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C48" s="46">
         <v>2106909869</v>
       </c>
       <c r="D48" s="47" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E48" s="20"/>
-      <c r="F48" s="48" t="s">
-        <v>172</v>
+      <c r="F48" s="53" t="s">
+        <v>166</v>
       </c>
       <c r="G48" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="H48" s="52">
-        <v>2</v>
-      </c>
+      <c r="H48" s="16"/>
       <c r="I48" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J48" s="16">
         <v>1.7909999999999999</v>
@@ -2733,16 +2737,16 @@
         <v>1.696</v>
       </c>
       <c r="L48" s="16">
-        <v>12.92</v>
+        <v>12.24</v>
       </c>
       <c r="M48" s="16" t="s">
         <v>40</v>
       </c>
       <c r="N48" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O48" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P48" s="48" t="s">
         <v>52</v>
@@ -2756,26 +2760,24 @@
         <v>4</v>
       </c>
       <c r="B49" s="45" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C49" s="46">
         <v>2106909869</v>
       </c>
       <c r="D49" s="47" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="E49" s="20"/>
-      <c r="F49" s="53" t="s">
-        <v>174</v>
+      <c r="F49" s="48" t="s">
+        <v>169</v>
       </c>
       <c r="G49" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="H49" s="16">
-        <v>6</v>
-      </c>
+      <c r="H49" s="16"/>
       <c r="I49" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J49" s="16">
         <v>1.7909999999999999</v>
@@ -2790,10 +2792,10 @@
         <v>40</v>
       </c>
       <c r="N49" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O49" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P49" s="48" t="s">
         <v>52</v>
@@ -2807,44 +2809,42 @@
         <v>5</v>
       </c>
       <c r="B50" s="45" t="s">
+        <v>170</v>
+      </c>
+      <c r="C50" s="46">
+        <v>2106909869</v>
+      </c>
+      <c r="D50" s="47" t="s">
         <v>156</v>
       </c>
-      <c r="C50" s="46">
-        <v>1905909060</v>
-      </c>
-      <c r="D50" s="47" t="s">
-        <v>157</v>
-      </c>
       <c r="E50" s="20"/>
-      <c r="F50" s="48" t="s">
-        <v>158</v>
+      <c r="F50" s="57" t="s">
+        <v>171</v>
       </c>
       <c r="G50" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="H50" s="16">
-        <v>0</v>
-      </c>
+      <c r="H50" s="52"/>
       <c r="I50" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J50" s="16">
-        <v>1.2</v>
+        <v>1.7909999999999999</v>
       </c>
       <c r="K50" s="16">
-        <v>1.1000000000000001</v>
+        <v>1.696</v>
       </c>
       <c r="L50" s="16">
-        <v>10.76</v>
+        <v>12.24</v>
       </c>
       <c r="M50" s="16" t="s">
         <v>40</v>
       </c>
       <c r="N50" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O50" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P50" s="48" t="s">
         <v>52</v>
@@ -2858,44 +2858,42 @@
         <v>6</v>
       </c>
       <c r="B51" s="45" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C51" s="46">
-        <v>2106909869</v>
+        <v>1905909060</v>
       </c>
       <c r="D51" s="47" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="E51" s="20"/>
-      <c r="F51" s="48" t="s">
-        <v>166</v>
+      <c r="F51" s="57" t="s">
+        <v>174</v>
       </c>
       <c r="G51" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="H51" s="52">
-        <v>2</v>
-      </c>
+      <c r="H51" s="52"/>
       <c r="I51" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J51" s="16">
-        <v>1.7909999999999999</v>
+        <v>1.2</v>
       </c>
       <c r="K51" s="16">
-        <v>1.696</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="L51" s="16">
-        <v>12.92</v>
+        <v>10.76</v>
       </c>
       <c r="M51" s="16" t="s">
         <v>40</v>
       </c>
       <c r="N51" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O51" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P51" s="48" t="s">
         <v>52</v>
@@ -2909,26 +2907,24 @@
         <v>7</v>
       </c>
       <c r="B52" s="45" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="C52" s="46">
         <v>1905909060</v>
       </c>
       <c r="D52" s="47" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E52" s="20"/>
-      <c r="F52" s="48" t="s">
-        <v>163</v>
+      <c r="F52" s="57" t="s">
+        <v>175</v>
       </c>
       <c r="G52" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="H52" s="52">
-        <v>8</v>
-      </c>
+      <c r="H52" s="52"/>
       <c r="I52" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J52" s="16">
         <v>1.2</v>
@@ -2943,10 +2939,10 @@
         <v>40</v>
       </c>
       <c r="N52" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="O52" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="P52" s="48" t="s">
         <v>52</v>
@@ -2957,7 +2953,7 @@
     </row>
     <row r="53" spans="1:19" ht="15.75" customHeight="1">
       <c r="A53" s="16">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B53" s="16"/>
       <c r="C53" s="16"/>
@@ -2965,7 +2961,7 @@
       <c r="E53" s="20"/>
       <c r="F53" s="48"/>
       <c r="G53" s="49"/>
-      <c r="H53" s="16"/>
+      <c r="H53" s="52"/>
       <c r="I53" s="16"/>
       <c r="J53" s="16"/>
       <c r="K53" s="16"/>
@@ -2980,15 +2976,15 @@
     </row>
     <row r="54" spans="1:19" ht="15.75" customHeight="1">
       <c r="A54" s="16">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B54" s="16"/>
       <c r="C54" s="16"/>
       <c r="D54" s="54"/>
       <c r="E54" s="20"/>
-      <c r="F54" s="48"/>
+      <c r="F54" s="16"/>
       <c r="G54" s="49"/>
-      <c r="H54" s="52"/>
+      <c r="H54" s="16"/>
       <c r="I54" s="16"/>
       <c r="J54" s="16"/>
       <c r="K54" s="16"/>
@@ -2996,22 +2992,22 @@
       <c r="M54" s="16"/>
       <c r="N54" s="16"/>
       <c r="O54" s="16"/>
-      <c r="P54" s="48"/>
+      <c r="P54" s="16"/>
       <c r="Q54" s="50"/>
       <c r="R54" s="20"/>
       <c r="S54" s="51"/>
     </row>
     <row r="55" spans="1:19" ht="15.75" customHeight="1">
       <c r="A55" s="16">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B55" s="16"/>
       <c r="C55" s="16"/>
       <c r="D55" s="54"/>
       <c r="E55" s="20"/>
-      <c r="F55" s="48"/>
+      <c r="F55" s="16"/>
       <c r="G55" s="49"/>
-      <c r="H55" s="52"/>
+      <c r="H55" s="16"/>
       <c r="I55" s="16"/>
       <c r="J55" s="16"/>
       <c r="K55" s="16"/>
@@ -3019,22 +3015,22 @@
       <c r="M55" s="16"/>
       <c r="N55" s="16"/>
       <c r="O55" s="16"/>
-      <c r="P55" s="48"/>
+      <c r="P55" s="16"/>
       <c r="Q55" s="50"/>
       <c r="R55" s="20"/>
       <c r="S55" s="51"/>
     </row>
     <row r="56" spans="1:19" ht="15.75" customHeight="1">
       <c r="A56" s="16">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
       <c r="D56" s="54"/>
       <c r="E56" s="20"/>
-      <c r="F56" s="48"/>
+      <c r="F56" s="16"/>
       <c r="G56" s="49"/>
-      <c r="H56" s="52"/>
+      <c r="H56" s="16"/>
       <c r="I56" s="16"/>
       <c r="J56" s="16"/>
       <c r="K56" s="16"/>
@@ -3042,22 +3038,22 @@
       <c r="M56" s="16"/>
       <c r="N56" s="16"/>
       <c r="O56" s="16"/>
-      <c r="P56" s="48"/>
+      <c r="P56" s="16"/>
       <c r="Q56" s="50"/>
       <c r="R56" s="20"/>
       <c r="S56" s="51"/>
     </row>
     <row r="57" spans="1:19" ht="15.75" customHeight="1">
       <c r="A57" s="16">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B57" s="16"/>
       <c r="C57" s="16"/>
       <c r="D57" s="54"/>
       <c r="E57" s="20"/>
-      <c r="F57" s="48"/>
+      <c r="F57" s="16"/>
       <c r="G57" s="49"/>
-      <c r="H57" s="52"/>
+      <c r="H57" s="16"/>
       <c r="I57" s="16"/>
       <c r="J57" s="16"/>
       <c r="K57" s="16"/>
@@ -3065,14 +3061,14 @@
       <c r="M57" s="16"/>
       <c r="N57" s="16"/>
       <c r="O57" s="16"/>
-      <c r="P57" s="48"/>
+      <c r="P57" s="16"/>
       <c r="Q57" s="50"/>
       <c r="R57" s="20"/>
       <c r="S57" s="51"/>
     </row>
     <row r="58" spans="1:19" ht="15.75" customHeight="1">
       <c r="A58" s="16">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B58" s="16"/>
       <c r="C58" s="16"/>
@@ -3095,7 +3091,7 @@
     </row>
     <row r="59" spans="1:19" ht="15.75" customHeight="1">
       <c r="A59" s="16">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B59" s="16"/>
       <c r="C59" s="16"/>
@@ -3118,7 +3114,7 @@
     </row>
     <row r="60" spans="1:19" ht="15.75" customHeight="1">
       <c r="A60" s="16">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B60" s="16"/>
       <c r="C60" s="16"/>
@@ -3141,13 +3137,13 @@
     </row>
     <row r="61" spans="1:19" ht="15.75" customHeight="1">
       <c r="A61" s="16">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="16"/>
       <c r="D61" s="54"/>
       <c r="E61" s="20"/>
-      <c r="F61" s="16"/>
+      <c r="F61" s="55"/>
       <c r="G61" s="49"/>
       <c r="H61" s="16"/>
       <c r="I61" s="16"/>
@@ -3164,13 +3160,13 @@
     </row>
     <row r="62" spans="1:19" ht="15.75" customHeight="1">
       <c r="A62" s="16">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="16"/>
       <c r="D62" s="54"/>
       <c r="E62" s="20"/>
-      <c r="F62" s="16"/>
+      <c r="F62" s="55"/>
       <c r="G62" s="49"/>
       <c r="H62" s="16"/>
       <c r="I62" s="16"/>
@@ -3187,13 +3183,13 @@
     </row>
     <row r="63" spans="1:19" ht="15.75" customHeight="1">
       <c r="A63" s="16">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B63" s="16"/>
       <c r="C63" s="16"/>
       <c r="D63" s="54"/>
       <c r="E63" s="20"/>
-      <c r="F63" s="16"/>
+      <c r="F63" s="55"/>
       <c r="G63" s="49"/>
       <c r="H63" s="16"/>
       <c r="I63" s="16"/>
@@ -3210,13 +3206,13 @@
     </row>
     <row r="64" spans="1:19" ht="15.75" customHeight="1">
       <c r="A64" s="16">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B64" s="16"/>
       <c r="C64" s="16"/>
       <c r="D64" s="54"/>
       <c r="E64" s="20"/>
-      <c r="F64" s="16"/>
+      <c r="F64" s="55"/>
       <c r="G64" s="49"/>
       <c r="H64" s="16"/>
       <c r="I64" s="16"/>
@@ -3233,7 +3229,7 @@
     </row>
     <row r="65" spans="1:19" ht="15.75" customHeight="1">
       <c r="A65" s="16">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B65" s="16"/>
       <c r="C65" s="16"/>
@@ -3256,7 +3252,7 @@
     </row>
     <row r="66" spans="1:19" ht="15.75" customHeight="1">
       <c r="A66" s="16">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B66" s="16"/>
       <c r="C66" s="16"/>
@@ -3279,7 +3275,7 @@
     </row>
     <row r="67" spans="1:19" ht="15.75" customHeight="1">
       <c r="A67" s="16">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B67" s="16"/>
       <c r="C67" s="16"/>
@@ -3302,7 +3298,7 @@
     </row>
     <row r="68" spans="1:19" ht="15.75" customHeight="1">
       <c r="A68" s="16">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B68" s="16"/>
       <c r="C68" s="16"/>
@@ -3325,7 +3321,7 @@
     </row>
     <row r="69" spans="1:19" ht="15.75" customHeight="1">
       <c r="A69" s="16">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B69" s="16"/>
       <c r="C69" s="16"/>
@@ -3348,7 +3344,7 @@
     </row>
     <row r="70" spans="1:19" ht="15.75" customHeight="1">
       <c r="A70" s="16">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B70" s="16"/>
       <c r="C70" s="16"/>
@@ -3371,7 +3367,7 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" customHeight="1">
       <c r="A71" s="16">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B71" s="16"/>
       <c r="C71" s="16"/>
@@ -3394,7 +3390,7 @@
     </row>
     <row r="72" spans="1:19" ht="15.75" customHeight="1">
       <c r="A72" s="16">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B72" s="16"/>
       <c r="C72" s="16"/>
@@ -3417,7 +3413,7 @@
     </row>
     <row r="73" spans="1:19" ht="15.75" customHeight="1">
       <c r="A73" s="16">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B73" s="16"/>
       <c r="C73" s="16"/>
@@ -3440,7 +3436,7 @@
     </row>
     <row r="74" spans="1:19" ht="15.75" customHeight="1">
       <c r="A74" s="16">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B74" s="16"/>
       <c r="C74" s="16"/>
@@ -3463,7 +3459,7 @@
     </row>
     <row r="75" spans="1:19" ht="15.75" customHeight="1">
       <c r="A75" s="16">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B75" s="16"/>
       <c r="C75" s="16"/>
@@ -3486,7 +3482,7 @@
     </row>
     <row r="76" spans="1:19" ht="15.75" customHeight="1">
       <c r="A76" s="16">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B76" s="16"/>
       <c r="C76" s="16"/>
@@ -3509,7 +3505,7 @@
     </row>
     <row r="77" spans="1:19" ht="15.75" customHeight="1">
       <c r="A77" s="16">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B77" s="16"/>
       <c r="C77" s="16"/>
@@ -3532,7 +3528,7 @@
     </row>
     <row r="78" spans="1:19" ht="15.75" customHeight="1">
       <c r="A78" s="16">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B78" s="16"/>
       <c r="C78" s="16"/>
@@ -3555,7 +3551,7 @@
     </row>
     <row r="79" spans="1:19" ht="15.75" customHeight="1">
       <c r="A79" s="16">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B79" s="16"/>
       <c r="C79" s="16"/>
@@ -3578,7 +3574,7 @@
     </row>
     <row r="80" spans="1:19" ht="15.75" customHeight="1">
       <c r="A80" s="16">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B80" s="16"/>
       <c r="C80" s="16"/>
@@ -3601,7 +3597,7 @@
     </row>
     <row r="81" spans="1:19" ht="15.75" customHeight="1">
       <c r="A81" s="16">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B81" s="16"/>
       <c r="C81" s="16"/>
@@ -3624,7 +3620,7 @@
     </row>
     <row r="82" spans="1:19" ht="15.75" customHeight="1">
       <c r="A82" s="16">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B82" s="16"/>
       <c r="C82" s="16"/>
@@ -3647,7 +3643,7 @@
     </row>
     <row r="83" spans="1:19" ht="15.75" customHeight="1">
       <c r="A83" s="16">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B83" s="16"/>
       <c r="C83" s="16"/>
@@ -3670,7 +3666,7 @@
     </row>
     <row r="84" spans="1:19" ht="15.75" customHeight="1">
       <c r="A84" s="16">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B84" s="16"/>
       <c r="C84" s="16"/>
@@ -3693,7 +3689,7 @@
     </row>
     <row r="85" spans="1:19" ht="15.75" customHeight="1">
       <c r="A85" s="16">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B85" s="16"/>
       <c r="C85" s="16"/>
@@ -3716,7 +3712,7 @@
     </row>
     <row r="86" spans="1:19" ht="15.75" customHeight="1">
       <c r="A86" s="16">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B86" s="16"/>
       <c r="C86" s="16"/>
@@ -3739,7 +3735,7 @@
     </row>
     <row r="87" spans="1:19" ht="15.75" customHeight="1">
       <c r="A87" s="16">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B87" s="16"/>
       <c r="C87" s="16"/>
@@ -3762,7 +3758,7 @@
     </row>
     <row r="88" spans="1:19" ht="15.75" customHeight="1">
       <c r="A88" s="16">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B88" s="16"/>
       <c r="C88" s="16"/>
@@ -3785,7 +3781,7 @@
     </row>
     <row r="89" spans="1:19" ht="15.75" customHeight="1">
       <c r="A89" s="16">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B89" s="16"/>
       <c r="C89" s="16"/>
@@ -3808,7 +3804,7 @@
     </row>
     <row r="90" spans="1:19" ht="15.75" customHeight="1">
       <c r="A90" s="16">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B90" s="16"/>
       <c r="C90" s="16"/>
@@ -3831,7 +3827,7 @@
     </row>
     <row r="91" spans="1:19" ht="15.75" customHeight="1">
       <c r="A91" s="16">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B91" s="16"/>
       <c r="C91" s="16"/>
@@ -3854,7 +3850,7 @@
     </row>
     <row r="92" spans="1:19" ht="15.75" customHeight="1">
       <c r="A92" s="16">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B92" s="16"/>
       <c r="C92" s="16"/>
@@ -3877,7 +3873,7 @@
     </row>
     <row r="93" spans="1:19" ht="15.75" customHeight="1">
       <c r="A93" s="16">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B93" s="16"/>
       <c r="C93" s="16"/>
@@ -3900,7 +3896,7 @@
     </row>
     <row r="94" spans="1:19" ht="15.75" customHeight="1">
       <c r="A94" s="16">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B94" s="16"/>
       <c r="C94" s="16"/>
@@ -3923,7 +3919,7 @@
     </row>
     <row r="95" spans="1:19" ht="15.75" customHeight="1">
       <c r="A95" s="16">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B95" s="16"/>
       <c r="C95" s="16"/>
@@ -3946,7 +3942,7 @@
     </row>
     <row r="96" spans="1:19" ht="15.75" customHeight="1">
       <c r="A96" s="16">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B96" s="16"/>
       <c r="C96" s="16"/>
@@ -3969,7 +3965,7 @@
     </row>
     <row r="97" spans="1:19" ht="15.75" customHeight="1">
       <c r="A97" s="16">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B97" s="16"/>
       <c r="C97" s="16"/>
@@ -3992,7 +3988,7 @@
     </row>
     <row r="98" spans="1:19" ht="15.75" customHeight="1">
       <c r="A98" s="16">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B98" s="16"/>
       <c r="C98" s="16"/>
@@ -4015,7 +4011,7 @@
     </row>
     <row r="99" spans="1:19" ht="15.75" customHeight="1">
       <c r="A99" s="16">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B99" s="16"/>
       <c r="C99" s="16"/>
@@ -4038,7 +4034,7 @@
     </row>
     <row r="100" spans="1:19" ht="15.75" customHeight="1">
       <c r="A100" s="16">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B100" s="16"/>
       <c r="C100" s="16"/>
@@ -4061,7 +4057,7 @@
     </row>
     <row r="101" spans="1:19" ht="15.75" customHeight="1">
       <c r="A101" s="16">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B101" s="16"/>
       <c r="C101" s="16"/>
@@ -4084,7 +4080,7 @@
     </row>
     <row r="102" spans="1:19" ht="15.75" customHeight="1">
       <c r="A102" s="16">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B102" s="16"/>
       <c r="C102" s="16"/>
@@ -4107,7 +4103,7 @@
     </row>
     <row r="103" spans="1:19" ht="15.75" customHeight="1">
       <c r="A103" s="16">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B103" s="16"/>
       <c r="C103" s="16"/>
@@ -4130,7 +4126,7 @@
     </row>
     <row r="104" spans="1:19" ht="15.75" customHeight="1">
       <c r="A104" s="16">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B104" s="16"/>
       <c r="C104" s="16"/>
@@ -4153,7 +4149,7 @@
     </row>
     <row r="105" spans="1:19" ht="15.75" customHeight="1">
       <c r="A105" s="16">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B105" s="16"/>
       <c r="C105" s="16"/>
@@ -4176,7 +4172,7 @@
     </row>
     <row r="106" spans="1:19" ht="15.75" customHeight="1">
       <c r="A106" s="16">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B106" s="16"/>
       <c r="C106" s="16"/>
@@ -4199,7 +4195,7 @@
     </row>
     <row r="107" spans="1:19" ht="15.75" customHeight="1">
       <c r="A107" s="16">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B107" s="16"/>
       <c r="C107" s="16"/>
@@ -4222,7 +4218,7 @@
     </row>
     <row r="108" spans="1:19" ht="15.75" customHeight="1">
       <c r="A108" s="16">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B108" s="16"/>
       <c r="C108" s="16"/>
@@ -4245,7 +4241,7 @@
     </row>
     <row r="109" spans="1:19" ht="15.75" customHeight="1">
       <c r="A109" s="16">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B109" s="16"/>
       <c r="C109" s="16"/>
@@ -4268,7 +4264,7 @@
     </row>
     <row r="110" spans="1:19" ht="15.75" customHeight="1">
       <c r="A110" s="16">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B110" s="16"/>
       <c r="C110" s="16"/>
@@ -4291,7 +4287,7 @@
     </row>
     <row r="111" spans="1:19" ht="15.75" customHeight="1">
       <c r="A111" s="16">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B111" s="16"/>
       <c r="C111" s="16"/>
@@ -4314,7 +4310,7 @@
     </row>
     <row r="112" spans="1:19" ht="15.75" customHeight="1">
       <c r="A112" s="16">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B112" s="16"/>
       <c r="C112" s="16"/>
@@ -4337,7 +4333,7 @@
     </row>
     <row r="113" spans="1:19" ht="15.75" customHeight="1">
       <c r="A113" s="16">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B113" s="16"/>
       <c r="C113" s="16"/>
@@ -4360,7 +4356,7 @@
     </row>
     <row r="114" spans="1:19" ht="15.75" customHeight="1">
       <c r="A114" s="16">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B114" s="16"/>
       <c r="C114" s="16"/>
@@ -4383,7 +4379,7 @@
     </row>
     <row r="115" spans="1:19" ht="15.75" customHeight="1">
       <c r="A115" s="16">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B115" s="16"/>
       <c r="C115" s="16"/>
@@ -4406,7 +4402,7 @@
     </row>
     <row r="116" spans="1:19" ht="15.75" customHeight="1">
       <c r="A116" s="16">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B116" s="16"/>
       <c r="C116" s="16"/>
@@ -4429,7 +4425,7 @@
     </row>
     <row r="117" spans="1:19" ht="15.75" customHeight="1">
       <c r="A117" s="16">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B117" s="16"/>
       <c r="C117" s="16"/>
@@ -4452,7 +4448,7 @@
     </row>
     <row r="118" spans="1:19" ht="15.75" customHeight="1">
       <c r="A118" s="16">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B118" s="16"/>
       <c r="C118" s="16"/>
@@ -4475,7 +4471,7 @@
     </row>
     <row r="119" spans="1:19" ht="15.75" customHeight="1">
       <c r="A119" s="16">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B119" s="16"/>
       <c r="C119" s="16"/>
@@ -4498,7 +4494,7 @@
     </row>
     <row r="120" spans="1:19" ht="15.75" customHeight="1">
       <c r="A120" s="16">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B120" s="16"/>
       <c r="C120" s="16"/>
@@ -4521,7 +4517,7 @@
     </row>
     <row r="121" spans="1:19" ht="15.75" customHeight="1">
       <c r="A121" s="16">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B121" s="16"/>
       <c r="C121" s="16"/>
@@ -4544,7 +4540,7 @@
     </row>
     <row r="122" spans="1:19" ht="15.75" customHeight="1">
       <c r="A122" s="16">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B122" s="16"/>
       <c r="C122" s="16"/>
@@ -4567,7 +4563,7 @@
     </row>
     <row r="123" spans="1:19" ht="15.75" customHeight="1">
       <c r="A123" s="16">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B123" s="16"/>
       <c r="C123" s="16"/>
@@ -4590,7 +4586,7 @@
     </row>
     <row r="124" spans="1:19" ht="15.75" customHeight="1">
       <c r="A124" s="16">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B124" s="16"/>
       <c r="C124" s="16"/>
@@ -4613,7 +4609,7 @@
     </row>
     <row r="125" spans="1:19" ht="15.75" customHeight="1">
       <c r="A125" s="16">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B125" s="16"/>
       <c r="C125" s="16"/>
@@ -4636,7 +4632,7 @@
     </row>
     <row r="126" spans="1:19" ht="15.75" customHeight="1">
       <c r="A126" s="16">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B126" s="16"/>
       <c r="C126" s="16"/>
@@ -4659,7 +4655,7 @@
     </row>
     <row r="127" spans="1:19" ht="15.75" customHeight="1">
       <c r="A127" s="16">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B127" s="16"/>
       <c r="C127" s="16"/>
@@ -4682,7 +4678,7 @@
     </row>
     <row r="128" spans="1:19" ht="15.75" customHeight="1">
       <c r="A128" s="16">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B128" s="16"/>
       <c r="C128" s="16"/>
@@ -4705,7 +4701,7 @@
     </row>
     <row r="129" spans="1:19" ht="15.75" customHeight="1">
       <c r="A129" s="16">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B129" s="16"/>
       <c r="C129" s="16"/>
@@ -4728,7 +4724,7 @@
     </row>
     <row r="130" spans="1:19" ht="15.75" customHeight="1">
       <c r="A130" s="16">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B130" s="16"/>
       <c r="C130" s="16"/>
@@ -4751,7 +4747,7 @@
     </row>
     <row r="131" spans="1:19" ht="15.75" customHeight="1">
       <c r="A131" s="16">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B131" s="16"/>
       <c r="C131" s="16"/>
@@ -4774,7 +4770,7 @@
     </row>
     <row r="132" spans="1:19" ht="15.75" customHeight="1">
       <c r="A132" s="16">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B132" s="16"/>
       <c r="C132" s="16"/>
@@ -4797,7 +4793,7 @@
     </row>
     <row r="133" spans="1:19" ht="15.75" customHeight="1">
       <c r="A133" s="16">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B133" s="16"/>
       <c r="C133" s="16"/>
@@ -4820,7 +4816,7 @@
     </row>
     <row r="134" spans="1:19" ht="15.75" customHeight="1">
       <c r="A134" s="16">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B134" s="16"/>
       <c r="C134" s="16"/>
@@ -4843,7 +4839,7 @@
     </row>
     <row r="135" spans="1:19" ht="15.75" customHeight="1">
       <c r="A135" s="16">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B135" s="16"/>
       <c r="C135" s="16"/>
@@ -4866,7 +4862,7 @@
     </row>
     <row r="136" spans="1:19" ht="15.75" customHeight="1">
       <c r="A136" s="16">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B136" s="16"/>
       <c r="C136" s="16"/>
@@ -4889,7 +4885,7 @@
     </row>
     <row r="137" spans="1:19" ht="15.75" customHeight="1">
       <c r="A137" s="16">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B137" s="16"/>
       <c r="C137" s="16"/>
@@ -4912,7 +4908,7 @@
     </row>
     <row r="138" spans="1:19" ht="15.75" customHeight="1">
       <c r="A138" s="16">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B138" s="16"/>
       <c r="C138" s="16"/>
@@ -4935,7 +4931,7 @@
     </row>
     <row r="139" spans="1:19" ht="15.75" customHeight="1">
       <c r="A139" s="16">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B139" s="16"/>
       <c r="C139" s="16"/>
@@ -4957,118 +4953,30 @@
       <c r="S139" s="51"/>
     </row>
     <row r="140" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A140" s="16">
-        <v>95</v>
-      </c>
-      <c r="B140" s="16"/>
-      <c r="C140" s="16"/>
-      <c r="D140" s="54"/>
-      <c r="E140" s="20"/>
-      <c r="F140" s="55"/>
-      <c r="G140" s="49"/>
-      <c r="H140" s="16"/>
+      <c r="A140" s="2"/>
+      <c r="B140" s="2"/>
+      <c r="C140" s="2"/>
+      <c r="D140" s="2"/>
+      <c r="E140" s="2"/>
+      <c r="F140" s="2"/>
+      <c r="G140" s="2"/>
+      <c r="H140" s="2"/>
       <c r="I140" s="16"/>
-      <c r="J140" s="16"/>
-      <c r="K140" s="16"/>
-      <c r="L140" s="16"/>
+      <c r="J140" s="2"/>
+      <c r="K140" s="2"/>
+      <c r="L140" s="2"/>
       <c r="M140" s="16"/>
-      <c r="N140" s="16"/>
-      <c r="O140" s="16"/>
-      <c r="P140" s="16"/>
-      <c r="Q140" s="50"/>
-      <c r="R140" s="20"/>
-      <c r="S140" s="51"/>
-    </row>
-    <row r="141" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A141" s="16">
-        <v>96</v>
-      </c>
-      <c r="B141" s="16"/>
-      <c r="C141" s="16"/>
-      <c r="D141" s="54"/>
-      <c r="E141" s="20"/>
-      <c r="F141" s="55"/>
-      <c r="G141" s="49"/>
-      <c r="H141" s="16"/>
-      <c r="I141" s="16"/>
-      <c r="J141" s="16"/>
-      <c r="K141" s="16"/>
-      <c r="L141" s="16"/>
-      <c r="M141" s="16"/>
-      <c r="N141" s="16"/>
-      <c r="O141" s="16"/>
-      <c r="P141" s="16"/>
-      <c r="Q141" s="50"/>
-      <c r="R141" s="20"/>
-      <c r="S141" s="51"/>
-    </row>
-    <row r="142" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A142" s="16">
-        <v>97</v>
-      </c>
-      <c r="B142" s="16"/>
-      <c r="C142" s="16"/>
-      <c r="D142" s="54"/>
-      <c r="E142" s="20"/>
-      <c r="F142" s="55"/>
-      <c r="G142" s="49"/>
-      <c r="H142" s="16"/>
-      <c r="I142" s="16"/>
-      <c r="J142" s="16"/>
-      <c r="K142" s="16"/>
-      <c r="L142" s="16"/>
-      <c r="M142" s="16"/>
-      <c r="N142" s="16"/>
-      <c r="O142" s="16"/>
-      <c r="P142" s="16"/>
-      <c r="Q142" s="50"/>
-      <c r="R142" s="20"/>
-      <c r="S142" s="51"/>
-    </row>
-    <row r="143" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A143" s="16">
-        <v>98</v>
-      </c>
-      <c r="B143" s="16"/>
-      <c r="C143" s="16"/>
-      <c r="D143" s="54"/>
-      <c r="E143" s="20"/>
-      <c r="F143" s="55"/>
-      <c r="G143" s="49"/>
-      <c r="H143" s="16"/>
-      <c r="I143" s="16"/>
-      <c r="J143" s="16"/>
-      <c r="K143" s="16"/>
-      <c r="L143" s="16"/>
-      <c r="M143" s="16"/>
-      <c r="N143" s="16"/>
-      <c r="O143" s="16"/>
-      <c r="P143" s="16"/>
-      <c r="Q143" s="50"/>
-      <c r="R143" s="20"/>
-      <c r="S143" s="51"/>
-    </row>
-    <row r="144" spans="1:19" ht="15.75" customHeight="1">
-      <c r="A144" s="2"/>
-      <c r="B144" s="2"/>
-      <c r="C144" s="2"/>
-      <c r="D144" s="2"/>
-      <c r="E144" s="2"/>
-      <c r="F144" s="2"/>
-      <c r="G144" s="2"/>
-      <c r="H144" s="2"/>
-      <c r="I144" s="16"/>
-      <c r="J144" s="2"/>
-      <c r="K144" s="2"/>
-      <c r="L144" s="2"/>
-      <c r="M144" s="16"/>
-      <c r="N144" s="2"/>
-      <c r="O144" s="2"/>
-      <c r="P144" s="2"/>
-      <c r="Q144" s="2"/>
-      <c r="R144" s="2"/>
-      <c r="S144" s="2"/>
-    </row>
+      <c r="N140" s="2"/>
+      <c r="O140" s="2"/>
+      <c r="P140" s="2"/>
+      <c r="Q140" s="2"/>
+      <c r="R140" s="2"/>
+      <c r="S140" s="2"/>
+    </row>
+    <row r="141" spans="1:19" ht="15.75" customHeight="1"/>
+    <row r="142" spans="1:19" ht="15.75" customHeight="1"/>
+    <row r="143" spans="1:19" ht="15.75" customHeight="1"/>
+    <row r="144" spans="1:19" ht="15.75" customHeight="1"/>
     <row r="145" ht="15.75" customHeight="1"/>
     <row r="146" ht="15.75" customHeight="1"/>
     <row r="147" ht="15.75" customHeight="1"/>
@@ -5920,10 +5828,6 @@
     <row r="993" ht="15.75" customHeight="1"/>
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A9:A42"/>
@@ -5939,17 +5843,18 @@
     <mergeCell ref="J32:L32"/>
     <mergeCell ref="K38:L38"/>
   </mergeCells>
+  <phoneticPr fontId="29" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="E19" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="E31" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="E45" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="D46" r:id="rId4" xr:uid="{0BBE21EA-B0B5-C344-AF08-088CCF395EF3}"/>
     <hyperlink ref="D47" r:id="rId5" xr:uid="{271E3DC7-0795-7E44-B144-E858EA3C3D4E}"/>
-    <hyperlink ref="D48" r:id="rId6" xr:uid="{7F4ECB7B-C689-F349-8AB3-0093A1BED64F}"/>
-    <hyperlink ref="D49" r:id="rId7" xr:uid="{784F22EF-BEC4-3140-BF64-7458A228E735}"/>
-    <hyperlink ref="D50" r:id="rId8" xr:uid="{B1BB5434-394D-C940-947D-AECA4099A6E7}"/>
-    <hyperlink ref="D51" r:id="rId9" xr:uid="{3977E940-0140-CA48-8F01-FCBD3B3EB23F}"/>
-    <hyperlink ref="D52" r:id="rId10" xr:uid="{21F67095-37E3-284B-9DC5-111BC028EB79}"/>
+    <hyperlink ref="D48" r:id="rId6" xr:uid="{784F22EF-BEC4-3140-BF64-7458A228E735}"/>
+    <hyperlink ref="D49" r:id="rId7" xr:uid="{5FB7BEEB-5649-3043-8680-BA5E3E5E750A}"/>
+    <hyperlink ref="D50" r:id="rId8" xr:uid="{DB28440C-A7B3-444F-8923-CF3811EF79AB}"/>
+    <hyperlink ref="D51" r:id="rId9" xr:uid="{F3C46BCE-132E-C041-A96F-027E5BF1D6D5}"/>
+    <hyperlink ref="D52" r:id="rId10" xr:uid="{624F99FC-99FF-E842-B60D-9A954F68749E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>